<commit_message>
Add Month_Order and Month_Label columns
</commit_message>
<xml_diff>
--- a/data/processed/monthly_summary.xlsx
+++ b/data/processed/monthly_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,269 +459,310 @@
           <t>Delay_Rate_%</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Month_Order</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Apr</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>253386</v>
+        <v>268120</v>
       </c>
       <c r="C2" t="n">
-        <v>42228</v>
+        <v>44465</v>
       </c>
       <c r="D2" t="n">
-        <v>3.53997627018094</v>
+        <v>2.190727994324827</v>
       </c>
       <c r="E2" t="n">
-        <v>75247936</v>
+        <v>83599428</v>
       </c>
       <c r="F2" t="n">
-        <v>16.7</v>
+        <v>16.6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Aug</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>286305</v>
+        <v>247964</v>
       </c>
       <c r="C3" t="n">
-        <v>55839</v>
+        <v>44521</v>
       </c>
       <c r="D3" t="n">
-        <v>6.453106345976344</v>
+        <v>3.712645778649035</v>
       </c>
       <c r="E3" t="n">
-        <v>103851970</v>
+        <v>79787170</v>
       </c>
       <c r="F3" t="n">
-        <v>19.5</v>
+        <v>18</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dec</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>214902</v>
+        <v>292564</v>
       </c>
       <c r="C4" t="n">
-        <v>43858</v>
+        <v>47259</v>
       </c>
       <c r="D4" t="n">
-        <v>6.67248358026577</v>
+        <v>2.255956087465131</v>
       </c>
       <c r="E4" t="n">
-        <v>83433002</v>
+        <v>83693186</v>
       </c>
       <c r="F4" t="n">
-        <v>20.4</v>
+        <v>16.2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>247964</v>
+        <v>253386</v>
       </c>
       <c r="C5" t="n">
-        <v>44521</v>
+        <v>42228</v>
       </c>
       <c r="D5" t="n">
-        <v>3.712645778649035</v>
+        <v>3.53997627018094</v>
       </c>
       <c r="E5" t="n">
-        <v>79787170</v>
+        <v>75247936</v>
       </c>
       <c r="F5" t="n">
-        <v>18</v>
+        <v>16.7</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>May</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>268120</v>
+        <v>251871</v>
       </c>
       <c r="C6" t="n">
-        <v>44465</v>
+        <v>42972</v>
       </c>
       <c r="D6" t="n">
-        <v>2.190727994324827</v>
+        <v>3.359410980487214</v>
       </c>
       <c r="E6" t="n">
-        <v>83599428</v>
+        <v>75411402</v>
       </c>
       <c r="F6" t="n">
-        <v>16.6</v>
+        <v>17.1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jul</t>
+          <t>Jun</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>284008</v>
+        <v>260254</v>
       </c>
       <c r="C7" t="n">
-        <v>62556</v>
+        <v>59327</v>
       </c>
       <c r="D7" t="n">
-        <v>9.491414824083668</v>
+        <v>10.06175342551706</v>
       </c>
       <c r="E7" t="n">
-        <v>119906048</v>
+        <v>110541940</v>
       </c>
       <c r="F7" t="n">
-        <v>22</v>
+        <v>22.8</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>Jul</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>260254</v>
+        <v>284008</v>
       </c>
       <c r="C8" t="n">
-        <v>59327</v>
+        <v>62556</v>
       </c>
       <c r="D8" t="n">
-        <v>10.06175342551706</v>
+        <v>9.491414824083668</v>
       </c>
       <c r="E8" t="n">
-        <v>110541940</v>
+        <v>119906048</v>
       </c>
       <c r="F8" t="n">
-        <v>22.8</v>
+        <v>22</v>
+      </c>
+      <c r="G8" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Aug</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>292564</v>
+        <v>286305</v>
       </c>
       <c r="C9" t="n">
-        <v>47259</v>
+        <v>55839</v>
       </c>
       <c r="D9" t="n">
-        <v>2.255956087465131</v>
+        <v>6.453106345976344</v>
       </c>
       <c r="E9" t="n">
-        <v>83693186</v>
+        <v>103851970</v>
       </c>
       <c r="F9" t="n">
-        <v>16.2</v>
+        <v>19.5</v>
+      </c>
+      <c r="G9" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Sep</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>251871</v>
+        <v>206535</v>
       </c>
       <c r="C10" t="n">
-        <v>42972</v>
+        <v>27198</v>
       </c>
       <c r="D10" t="n">
-        <v>3.359410980487214</v>
+        <v>-0.5121811252642473</v>
       </c>
       <c r="E10" t="n">
-        <v>75411402</v>
+        <v>49895832</v>
       </c>
       <c r="F10" t="n">
-        <v>17.1</v>
+        <v>13.2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Nov</t>
+          <t>Oct</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>210612</v>
+        <v>216407</v>
       </c>
       <c r="C11" t="n">
-        <v>30528</v>
+        <v>33112</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1641540317022743</v>
+        <v>1.424035878629324</v>
       </c>
       <c r="E11" t="n">
-        <v>55034244</v>
+        <v>57726882</v>
       </c>
       <c r="F11" t="n">
-        <v>14.5</v>
+        <v>15.3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Oct</t>
+          <t>Nov</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>216407</v>
+        <v>210612</v>
       </c>
       <c r="C12" t="n">
-        <v>33112</v>
+        <v>30528</v>
       </c>
       <c r="D12" t="n">
-        <v>1.424035878629324</v>
+        <v>0.1641540317022743</v>
       </c>
       <c r="E12" t="n">
-        <v>57726882</v>
+        <v>55034244</v>
       </c>
       <c r="F12" t="n">
-        <v>15.3</v>
+        <v>14.5</v>
+      </c>
+      <c r="G12" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sep</t>
+          <t>Dec</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>206535</v>
+        <v>214902</v>
       </c>
       <c r="C13" t="n">
-        <v>27198</v>
+        <v>43858</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.5121811252642473</v>
+        <v>6.67248358026577</v>
       </c>
       <c r="E13" t="n">
-        <v>49895832</v>
+        <v>83433002</v>
       </c>
       <c r="F13" t="n">
-        <v>13.2</v>
+        <v>20.4</v>
+      </c>
+      <c r="G13" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>